<commit_message>
Vamos a meter optimizaciones
</commit_message>
<xml_diff>
--- a/EstadisticasPlanificador_1.xlsx
+++ b/EstadisticasPlanificador_1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedre\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedre\Desktop\Planificador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAFB294D-0BC3-459A-A0B4-DF1A05FF3819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{819D1DC3-EF38-46E0-BDF8-771D0551CB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -151,8 +151,6 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -339,7 +337,7 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="13"/>
-                <c:pt idx="0">
+                <c:pt idx="0" formatCode="General">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
@@ -385,10 +383,10 @@
             <c:numRef>
               <c:f>Sheet1!$C$6:$C$18</c:f>
               <c:numCache>
-                <c:formatCode>0,000</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>7.2999999999999995E-2</c:v>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>6.0000000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.4E-2</c:v>
@@ -437,7 +435,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -469,7 +466,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -528,7 +525,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0,000" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -772,22 +769,22 @@
                 <c:pt idx="3" formatCode="General">
                   <c:v>271.40899999999999</c:v>
                 </c:pt>
-                <c:pt idx="4" formatCode="#,##0">
+                <c:pt idx="4" formatCode="#,##0.000">
                   <c:v>270.09300000000002</c:v>
                 </c:pt>
-                <c:pt idx="5" formatCode="#,##0">
+                <c:pt idx="5" formatCode="#,##0.000">
                   <c:v>270.06299999999999</c:v>
                 </c:pt>
-                <c:pt idx="6" formatCode="#,##0">
+                <c:pt idx="6" formatCode="#,##0.000">
                   <c:v>270.05399999999997</c:v>
                 </c:pt>
-                <c:pt idx="7" formatCode="#,##0">
+                <c:pt idx="7" formatCode="#,##0.000">
                   <c:v>271.13400000000001</c:v>
                 </c:pt>
-                <c:pt idx="8" formatCode="#,##0">
+                <c:pt idx="8" formatCode="#,##0.000">
                   <c:v>270.05099999999999</c:v>
                 </c:pt>
-                <c:pt idx="9" formatCode="#,##0">
+                <c:pt idx="9" formatCode="#,##0.000">
                   <c:v>5.1390000000000002</c:v>
                 </c:pt>
               </c:numCache>
@@ -839,8 +836,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -1136,13 +1134,13 @@
                 <c:pt idx="1">
                   <c:v>0.20599999999999999</c:v>
                 </c:pt>
-                <c:pt idx="2" formatCode="0,000">
+                <c:pt idx="2" formatCode="0.000">
                   <c:v>2.8450000000000002</c:v>
                 </c:pt>
-                <c:pt idx="3" formatCode="0,000">
+                <c:pt idx="3" formatCode="0.000">
                   <c:v>1.3959999999999999</c:v>
                 </c:pt>
-                <c:pt idx="4" formatCode="0,000">
+                <c:pt idx="4" formatCode="0.000">
                   <c:v>0.30299999999999999</c:v>
                 </c:pt>
               </c:numCache>
@@ -1616,8 +1614,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -1947,8 +1946,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -2296,8 +2296,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -2747,8 +2748,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -3072,8 +3074,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -3595,10 +3598,10 @@
                 <c:pt idx="1">
                   <c:v>0.51300000000000001</c:v>
                 </c:pt>
-                <c:pt idx="2" formatCode="#.##0000">
+                <c:pt idx="2" formatCode="#,##0.000">
                   <c:v>61.171999999999997</c:v>
                 </c:pt>
-                <c:pt idx="3" formatCode="#.##0000">
+                <c:pt idx="3" formatCode="#,##0.000">
                   <c:v>270.02699999999999</c:v>
                 </c:pt>
               </c:numCache>
@@ -3650,8 +3653,9 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
+            <a:round/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -9299,16 +9303,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
       <xdr:row>50</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -9638,19 +9642,19 @@
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="3:12" x14ac:dyDescent="0.25">
-      <c r="C6" s="7">
-        <v>7.2999999999999995E-2</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="C6" s="2">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="2">
         <v>1</v>
       </c>
       <c r="F6" s="2">
         <v>12</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <v>15</v>
       </c>
       <c r="K6" s="5"/>
@@ -10035,16 +10039,16 @@
       <c r="C33" s="8">
         <v>0.1</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="2">
         <v>1</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="2">
         <v>40</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="2">
         <v>60</v>
       </c>
     </row>
@@ -10053,152 +10057,152 @@
       <c r="C34" s="8">
         <v>14.08</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="2">
         <v>2</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="2">
         <v>40</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="2">
         <v>120</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C35" s="13">
+      <c r="C35" s="2">
         <v>270.14400000000001</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="2">
         <v>3</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="2">
         <v>40</v>
       </c>
-      <c r="G35">
+      <c r="G35" s="2">
         <v>180</v>
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C36" s="13">
+      <c r="C36" s="2">
         <v>271.40899999999999</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="2">
         <v>4</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="2">
         <v>40</v>
       </c>
-      <c r="G36">
+      <c r="G36" s="2">
         <v>240</v>
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="12">
+      <c r="C37" s="11">
         <v>270.09300000000002</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="2">
         <v>5</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="2">
         <v>40</v>
       </c>
-      <c r="G37">
+      <c r="G37" s="2">
         <v>300</v>
       </c>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="12">
+      <c r="C38" s="11">
         <v>270.06299999999999</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="2">
         <v>6</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="2">
         <v>40</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="2">
         <v>360</v>
       </c>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C39" s="12">
+      <c r="C39" s="11">
         <v>270.05399999999997</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="2">
         <v>7</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="2">
         <v>40</v>
       </c>
-      <c r="G39">
+      <c r="G39" s="2">
         <v>420</v>
       </c>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C40" s="12">
+      <c r="C40" s="11">
         <v>271.13400000000001</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E40">
+      <c r="E40" s="2">
         <v>8</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="2">
         <v>40</v>
       </c>
-      <c r="G40">
+      <c r="G40" s="2">
         <v>480</v>
       </c>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C41" s="12">
+      <c r="C41" s="11">
         <v>270.05099999999999</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="2">
         <v>9</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="2">
         <v>40</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="2">
         <v>540</v>
       </c>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C42" s="12">
+      <c r="C42" s="11">
         <v>5.1390000000000002</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="2">
         <v>10</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="2">
         <v>40</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="2">
         <v>600</v>
       </c>
     </row>

</xml_diff>